<commit_message>
Squeez squeez & Booking
</commit_message>
<xml_diff>
--- a/data/golfData.xlsx
+++ b/data/golfData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AMIT\squeez-playwright\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D93D019C-8C87-4379-BECC-269C94F226C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1097E566-4EB7-4632-9829-8A9AA00D1F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="3450" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="golfData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="133">
   <si>
     <t>name</t>
   </si>
@@ -382,66 +382,6 @@
     <t>https://booking20.com</t>
   </si>
   <si>
-    <t>+1 555-123-0001</t>
-  </si>
-  <si>
-    <t>+1 555-123-0002</t>
-  </si>
-  <si>
-    <t>+1 555-123-0003</t>
-  </si>
-  <si>
-    <t>+1 555-123-0004</t>
-  </si>
-  <si>
-    <t>+1 555-123-0005</t>
-  </si>
-  <si>
-    <t>+1 555-123-0006</t>
-  </si>
-  <si>
-    <t>+1 555-123-0007</t>
-  </si>
-  <si>
-    <t>+1 555-123-0008</t>
-  </si>
-  <si>
-    <t>+1 555-123-0009</t>
-  </si>
-  <si>
-    <t>+1 555-123-0010</t>
-  </si>
-  <si>
-    <t>+1 555-123-0011</t>
-  </si>
-  <si>
-    <t>+1 555-123-0012</t>
-  </si>
-  <si>
-    <t>+1 555-123-0013</t>
-  </si>
-  <si>
-    <t>+1 555-123-0014</t>
-  </si>
-  <si>
-    <t>+1 555-123-0015</t>
-  </si>
-  <si>
-    <t>+1 555-123-0016</t>
-  </si>
-  <si>
-    <t>+1 555-123-0017</t>
-  </si>
-  <si>
-    <t>+1 555-123-0018</t>
-  </si>
-  <si>
-    <t>+1 555-123-0019</t>
-  </si>
-  <si>
-    <t>+1 555-123-0020</t>
-  </si>
-  <si>
     <t>Florida</t>
   </si>
   <si>
@@ -473,13 +413,19 @@
   </si>
   <si>
     <t>interval</t>
+  </si>
+  <si>
+    <t>waitlistUnit</t>
+  </si>
+  <si>
+    <t>waitlistAmount</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -524,6 +470,12 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -564,7 +516,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -576,6 +528,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -881,7 +836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X21"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -894,6 +849,7 @@
     <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.85546875" customWidth="1"/>
     <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -901,9 +857,11 @@
     <col min="21" max="21" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.7109375" customWidth="1"/>
+    <col min="27" max="27" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -959,30 +917,36 @@
         <v>17</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>149</v>
+        <v>129</v>
+      </c>
+      <c r="Z1" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>38</v>
@@ -1003,13 +967,13 @@
         <v>60</v>
       </c>
       <c r="I2" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J2" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K2" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L2" t="s">
         <v>80</v>
@@ -1017,8 +981,8 @@
       <c r="M2" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="N2" t="s">
-        <v>120</v>
+      <c r="N2">
+        <v>8596321058</v>
       </c>
       <c r="O2">
         <v>51</v>
@@ -1036,27 +1000,33 @@
         <v>10</v>
       </c>
       <c r="T2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X2" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z2">
+        <v>5</v>
+      </c>
+      <c r="AA2">
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>38</v>
@@ -1077,13 +1047,13 @@
         <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J3" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K3" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L3" t="s">
         <v>81</v>
@@ -1091,8 +1061,8 @@
       <c r="M3" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="N3" t="s">
-        <v>121</v>
+      <c r="N3">
+        <v>8596321058</v>
       </c>
       <c r="O3">
         <v>52</v>
@@ -1110,27 +1080,33 @@
         <v>10</v>
       </c>
       <c r="T3" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U3" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V3" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W3" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X3" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z3">
+        <v>5</v>
+      </c>
+      <c r="AA3">
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>38</v>
@@ -1151,13 +1127,13 @@
         <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J4" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K4" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L4" t="s">
         <v>82</v>
@@ -1165,8 +1141,8 @@
       <c r="M4" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="N4" t="s">
-        <v>122</v>
+      <c r="N4">
+        <v>8596321058</v>
       </c>
       <c r="O4">
         <v>53</v>
@@ -1184,27 +1160,33 @@
         <v>10</v>
       </c>
       <c r="T4" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U4" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V4" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W4" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X4" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z4">
+        <v>5</v>
+      </c>
+      <c r="AA4">
+        <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>38</v>
@@ -1225,13 +1207,13 @@
         <v>63</v>
       </c>
       <c r="I5" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J5" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K5" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L5" t="s">
         <v>83</v>
@@ -1239,8 +1221,8 @@
       <c r="M5" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="N5" t="s">
-        <v>123</v>
+      <c r="N5">
+        <v>8596321058</v>
       </c>
       <c r="O5">
         <v>54</v>
@@ -1258,27 +1240,33 @@
         <v>10</v>
       </c>
       <c r="T5" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U5" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V5" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W5" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X5" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z5">
+        <v>5</v>
+      </c>
+      <c r="AA5">
+        <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>38</v>
@@ -1299,13 +1287,13 @@
         <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J6" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K6" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L6" t="s">
         <v>84</v>
@@ -1313,8 +1301,8 @@
       <c r="M6" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="N6" t="s">
-        <v>124</v>
+      <c r="N6">
+        <v>8596321058</v>
       </c>
       <c r="O6">
         <v>55</v>
@@ -1332,27 +1320,33 @@
         <v>10</v>
       </c>
       <c r="T6" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U6" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V6" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W6" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X6" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z6">
+        <v>5</v>
+      </c>
+      <c r="AA6">
+        <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>38</v>
@@ -1373,13 +1367,13 @@
         <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J7" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K7" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L7" t="s">
         <v>85</v>
@@ -1387,8 +1381,8 @@
       <c r="M7" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="N7" t="s">
-        <v>125</v>
+      <c r="N7">
+        <v>8596321058</v>
       </c>
       <c r="O7">
         <v>56</v>
@@ -1406,27 +1400,33 @@
         <v>10</v>
       </c>
       <c r="T7" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U7" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V7" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W7" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X7" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z7">
+        <v>5</v>
+      </c>
+      <c r="AA7">
+        <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>38</v>
@@ -1447,13 +1447,13 @@
         <v>66</v>
       </c>
       <c r="I8" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J8" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K8" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L8" t="s">
         <v>86</v>
@@ -1461,8 +1461,8 @@
       <c r="M8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="N8" t="s">
-        <v>126</v>
+      <c r="N8">
+        <v>8596321058</v>
       </c>
       <c r="O8">
         <v>57</v>
@@ -1480,27 +1480,33 @@
         <v>10</v>
       </c>
       <c r="T8" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U8" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V8" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W8" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X8" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z8">
+        <v>5</v>
+      </c>
+      <c r="AA8">
+        <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>25</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>38</v>
@@ -1521,13 +1527,13 @@
         <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J9" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K9" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L9" t="s">
         <v>87</v>
@@ -1535,8 +1541,8 @@
       <c r="M9" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="N9" t="s">
-        <v>127</v>
+      <c r="N9">
+        <v>8596321058</v>
       </c>
       <c r="O9">
         <v>58</v>
@@ -1554,27 +1560,33 @@
         <v>10</v>
       </c>
       <c r="T9" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U9" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V9" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W9" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X9" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z9">
+        <v>5</v>
+      </c>
+      <c r="AA9">
+        <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>38</v>
@@ -1595,13 +1607,13 @@
         <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J10" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K10" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L10" t="s">
         <v>88</v>
@@ -1609,8 +1621,8 @@
       <c r="M10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="N10" t="s">
-        <v>128</v>
+      <c r="N10">
+        <v>8596321058</v>
       </c>
       <c r="O10">
         <v>59</v>
@@ -1628,27 +1640,33 @@
         <v>10</v>
       </c>
       <c r="T10" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U10" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V10" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W10" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X10" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z10">
+        <v>5</v>
+      </c>
+      <c r="AA10">
+        <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>38</v>
@@ -1669,13 +1687,13 @@
         <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J11" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K11" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L11" t="s">
         <v>89</v>
@@ -1683,8 +1701,8 @@
       <c r="M11" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="N11" t="s">
-        <v>129</v>
+      <c r="N11">
+        <v>8596321058</v>
       </c>
       <c r="O11">
         <v>60</v>
@@ -1702,27 +1720,33 @@
         <v>10</v>
       </c>
       <c r="T11" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U11" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V11" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W11" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X11" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z11">
+        <v>5</v>
+      </c>
+      <c r="AA11">
+        <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>38</v>
@@ -1743,13 +1767,13 @@
         <v>70</v>
       </c>
       <c r="I12" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J12" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K12" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L12" t="s">
         <v>90</v>
@@ -1757,8 +1781,8 @@
       <c r="M12" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N12" t="s">
-        <v>130</v>
+      <c r="N12">
+        <v>8596321058</v>
       </c>
       <c r="O12">
         <v>61</v>
@@ -1776,27 +1800,33 @@
         <v>10</v>
       </c>
       <c r="T12" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U12" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V12" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W12" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X12" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z12">
+        <v>5</v>
+      </c>
+      <c r="AA12">
+        <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>38</v>
@@ -1817,13 +1847,13 @@
         <v>71</v>
       </c>
       <c r="I13" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J13" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K13" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L13" t="s">
         <v>91</v>
@@ -1831,8 +1861,8 @@
       <c r="M13" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="N13" t="s">
-        <v>131</v>
+      <c r="N13">
+        <v>8596321058</v>
       </c>
       <c r="O13">
         <v>62</v>
@@ -1850,27 +1880,33 @@
         <v>10</v>
       </c>
       <c r="T13" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U13" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V13" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W13" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X13" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z13">
+        <v>5</v>
+      </c>
+      <c r="AA13">
+        <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>38</v>
@@ -1891,13 +1927,13 @@
         <v>72</v>
       </c>
       <c r="I14" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J14" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K14" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L14" t="s">
         <v>92</v>
@@ -1905,8 +1941,8 @@
       <c r="M14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="N14" t="s">
-        <v>132</v>
+      <c r="N14">
+        <v>8596321058</v>
       </c>
       <c r="O14">
         <v>63</v>
@@ -1924,27 +1960,33 @@
         <v>10</v>
       </c>
       <c r="T14" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U14" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V14" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W14" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X14" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z14">
+        <v>5</v>
+      </c>
+      <c r="AA14">
+        <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>38</v>
@@ -1965,13 +2007,13 @@
         <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J15" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K15" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L15" t="s">
         <v>93</v>
@@ -1979,8 +2021,8 @@
       <c r="M15" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="N15" t="s">
-        <v>133</v>
+      <c r="N15">
+        <v>8596321058</v>
       </c>
       <c r="O15">
         <v>64</v>
@@ -1998,27 +2040,33 @@
         <v>10</v>
       </c>
       <c r="T15" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U15" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V15" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W15" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X15" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z15">
+        <v>5</v>
+      </c>
+      <c r="AA15">
+        <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>38</v>
@@ -2039,13 +2087,13 @@
         <v>74</v>
       </c>
       <c r="I16" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J16" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K16" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L16" t="s">
         <v>94</v>
@@ -2053,8 +2101,8 @@
       <c r="M16" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="N16" t="s">
-        <v>134</v>
+      <c r="N16">
+        <v>8596321058</v>
       </c>
       <c r="O16">
         <v>65</v>
@@ -2072,27 +2120,33 @@
         <v>10</v>
       </c>
       <c r="T16" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U16" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V16" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W16" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X16" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z16">
+        <v>5</v>
+      </c>
+      <c r="AA16">
+        <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>38</v>
@@ -2113,13 +2167,13 @@
         <v>75</v>
       </c>
       <c r="I17" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J17" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K17" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L17" t="s">
         <v>95</v>
@@ -2127,8 +2181,8 @@
       <c r="M17" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="N17" t="s">
-        <v>135</v>
+      <c r="N17">
+        <v>8596321058</v>
       </c>
       <c r="O17">
         <v>66</v>
@@ -2146,27 +2200,33 @@
         <v>10</v>
       </c>
       <c r="T17" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U17" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V17" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W17" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X17" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z17">
+        <v>5</v>
+      </c>
+      <c r="AA17">
+        <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>38</v>
@@ -2187,13 +2247,13 @@
         <v>76</v>
       </c>
       <c r="I18" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J18" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K18" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L18" t="s">
         <v>96</v>
@@ -2201,8 +2261,8 @@
       <c r="M18" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="N18" t="s">
-        <v>136</v>
+      <c r="N18">
+        <v>8596321058</v>
       </c>
       <c r="O18">
         <v>67</v>
@@ -2220,27 +2280,33 @@
         <v>10</v>
       </c>
       <c r="T18" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U18" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V18" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W18" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X18" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z18">
+        <v>5</v>
+      </c>
+      <c r="AA18">
+        <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>35</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>38</v>
@@ -2261,13 +2327,13 @@
         <v>77</v>
       </c>
       <c r="I19" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J19" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K19" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L19" t="s">
         <v>97</v>
@@ -2275,8 +2341,8 @@
       <c r="M19" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="N19" t="s">
-        <v>137</v>
+      <c r="N19">
+        <v>8596321058</v>
       </c>
       <c r="O19">
         <v>68</v>
@@ -2294,27 +2360,33 @@
         <v>10</v>
       </c>
       <c r="T19" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U19" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V19" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W19" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X19" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z19">
+        <v>5</v>
+      </c>
+      <c r="AA19">
+        <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>36</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>38</v>
@@ -2335,13 +2407,13 @@
         <v>78</v>
       </c>
       <c r="I20" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J20" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K20" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L20" t="s">
         <v>98</v>
@@ -2349,8 +2421,8 @@
       <c r="M20" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="N20" t="s">
-        <v>138</v>
+      <c r="N20">
+        <v>8596321058</v>
       </c>
       <c r="O20">
         <v>69</v>
@@ -2368,27 +2440,33 @@
         <v>10</v>
       </c>
       <c r="T20" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U20" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V20" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W20" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X20" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z20">
+        <v>5</v>
+      </c>
+      <c r="AA20">
+        <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>38</v>
@@ -2409,13 +2487,13 @@
         <v>79</v>
       </c>
       <c r="I21" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J21" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="K21" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="L21" t="s">
         <v>99</v>
@@ -2423,8 +2501,8 @@
       <c r="M21" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="N21" t="s">
-        <v>139</v>
+      <c r="N21">
+        <v>8596321058</v>
       </c>
       <c r="O21">
         <v>70</v>
@@ -2442,19 +2520,25 @@
         <v>10</v>
       </c>
       <c r="T21" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U21" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V21" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W21" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="X21" t="s">
-        <v>145</v>
+        <v>125</v>
+      </c>
+      <c r="Z21">
+        <v>5</v>
+      </c>
+      <c r="AA21">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>